<commit_message>
feat: añadir campo ascensor a ficha de vivienda
</commit_message>
<xml_diff>
--- a/COMPARABLE_FICHA_v4.xlsx
+++ b/COMPARABLE_FICHA_v4.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://galisteoortega.sharepoint.com/sites/CITAEARQUITECTURA/Documentos compartidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{C7F2A014-6AEB-4B60-9E83-74072B03B33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F20FE0AF-7F5D-4F75-9C11-6E4B0EEB5F0E}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="13_ncr:1_{C7F2A014-6AEB-4B60-9E83-74072B03B33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCD8D9C7-2D0A-4056-A4C3-21C83E861EF9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COMPARABLE 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>COMPARABLE 1</t>
   </si>
@@ -104,6 +107,9 @@
     <t>Vistas</t>
   </si>
   <si>
+    <t>Observaciones:</t>
+  </si>
+  <si>
     <t>Precio oferta (€)</t>
   </si>
   <si>
@@ -128,7 +134,7 @@
     <t>URL del anuncio</t>
   </si>
   <si>
-    <t>Observaciones:</t>
+    <t>Ascensor</t>
   </si>
 </sst>
 </file>
@@ -177,7 +183,7 @@
       <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -201,18 +207,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor rgb="FFE26B0A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE26B0A"/>
+        <fgColor rgb="FFEFEFEF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -492,17 +504,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -614,6 +615,45 @@
       </top>
       <bottom style="medium">
         <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -621,7 +661,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -668,80 +708,84 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1061,6 +1105,11 @@
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
 </we:webextension>
 </file>
 
@@ -1079,24 +1128,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
       <c r="E2" s="8" t="s">
         <v>2</v>
       </c>
@@ -1104,7 +1153,7 @@
       <c r="G2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="41" t="s">
+      <c r="H2" s="24" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1130,13 +1179,13 @@
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="18"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="36"/>
     </row>
     <row r="5" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
@@ -1182,93 +1231,95 @@
       <c r="C7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12" t="s">
+      <c r="D7" s="23"/>
+      <c r="E7" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="11"/>
+      <c r="F7" s="23"/>
       <c r="G7" s="12" t="s">
         <v>21</v>
       </c>
       <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="43"/>
+      <c r="E8" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="47"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="27"/>
     </row>
     <row r="9" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="29" t="s">
+      <c r="A9" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="29" t="s">
+      <c r="B9" s="19"/>
+      <c r="C9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="30">
+      <c r="D9" s="42"/>
+      <c r="E9" s="44" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="46">
         <v>0.08</v>
       </c>
-      <c r="G9" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="31">
+      <c r="G9" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="21">
         <f>(B9-D9)*(1-F9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="35" t="str">
+      <c r="A10" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="40"/>
+      <c r="H10" s="22" t="str">
         <f>IFERROR(H9/B6,"")</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="29" t="s">
+      <c r="A11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="38"/>
-      <c r="H11" s="39"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="28"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="30"/>
     </row>
     <row r="12" spans="1:8" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="45"/>
+        <v>31</v>
+      </c>
+      <c r="B12" s="25"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="27"/>
     </row>
     <row r="13" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1279,11 +1330,11 @@
     <mergeCell ref="D11:H11"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="D8:H8"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="F8:H8"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" sqref="H6" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Muy malo,Malo,Medio,Bueno,Muy bueno"</formula1>
     </dataValidation>
@@ -1296,12 +1347,26 @@
     <dataValidation type="list" allowBlank="1" sqref="F2:F3" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>""</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{FCB69D13-F5EB-4DD7-8A1C-9BA191FFA608}">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8c4cda04-322f-4194-a39e-32a54e031a6b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4764f0f6-458f-4af1-86bb-e0284dd86230">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1310,10 +1375,11 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010097CA67C2628CE54F8D866AAA67C10195" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="3afb9dcfc5bce065561282d928f850df">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4764f0f6-458f-4af1-86bb-e0284dd86230" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9c410835c732efb4c66379aed7270c67" ns2:_="">
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010097CA67C2628CE54F8D866AAA67C10195" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="f6521879415ec61b3e2a36a86657071d">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4764f0f6-458f-4af1-86bb-e0284dd86230" xmlns:ns3="8c4cda04-322f-4194-a39e-32a54e031a6b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="06429c3fc6c72fa55ca9eecdf29eab89" ns2:_="" ns3:_="">
     <xsd:import namespace="4764f0f6-458f-4af1-86bb-e0284dd86230"/>
+    <xsd:import namespace="8c4cda04-322f-4194-a39e-32a54e031a6b"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -1323,6 +1389,12 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1347,6 +1419,50 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="ad9aa05d-899f-4bcd-bc34-ca30d8e8bd5a" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8c4cda04-322f-4194-a39e-32a54e031a6b" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{12556f10-8dee-4f6c-8c53-993362e14be9}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="8c4cda04-322f-4194-a39e-32a54e031a6b">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -1448,13 +1564,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D457D60E-2D65-4661-A2EE-5F478299EE99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8c4cda04-322f-4194-a39e-32a54e031a6b"/>
+    <ds:schemaRef ds:uri="4764f0f6-458f-4af1-86bb-e0284dd86230"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{233941E5-26F6-4DDC-9E4A-513A54871FB5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1462,14 +1583,15 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C09DA889-6B2F-43B1-9D78-767C94DCDB6D}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAED7987-4CD6-494F-A0C1-E2C355DF8106}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="4764f0f6-458f-4af1-86bb-e0284dd86230"/>
+    <ds:schemaRef ds:uri="8c4cda04-322f-4194-a39e-32a54e031a6b"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -1478,13 +1600,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D457D60E-2D65-4661-A2EE-5F478299EE99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>